<commit_message>
publish pork retail Excel 2026-09-12
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-09-12</t>
+          <t>越南猪肉零售价格日报｜2026-09-13</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 06:32。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 06:23。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>10条在售商品</t>
+          <t>9条在售商品</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O14"/>
+  <dimension ref="A1:O13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-09-12</t>
+          <t>越南猪肉零售明细｜2026-09-13</t>
         </is>
       </c>
     </row>
@@ -1066,7 +1066,7 @@
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
+          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g-ol341387</t>
         </is>
       </c>
     </row>
@@ -1296,12 +1296,12 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>肩肉</t>
+          <t>小排</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI Thịt Nạc vai heo (S)</t>
+          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
@@ -1310,13 +1310,13 @@
         </is>
       </c>
       <c r="I12" s="7" t="n">
-        <v>440</v>
+        <v>431</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>74316</v>
+        <v>124085</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>168900</v>
+        <v>287900</v>
       </c>
       <c r="L12" s="7" t="n"/>
       <c r="M12" s="7">
@@ -1330,7 +1330,7 @@
       </c>
       <c r="O12" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-nac-vai-heo-s--s10140279</t>
+          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
         </is>
       </c>
     </row>
@@ -1362,12 +1362,12 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>小排</t>
+          <t>五花肉</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
+          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
@@ -1376,13 +1376,13 @@
         </is>
       </c>
       <c r="I13" s="7" t="n">
-        <v>431</v>
+        <v>385</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>124085</v>
+        <v>76962</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>287900</v>
+        <v>199900</v>
       </c>
       <c r="L13" s="7" t="n"/>
       <c r="M13" s="7">
@@ -1395,72 +1395,6 @@
         </is>
       </c>
       <c r="O13" s="8" t="inlineStr">
-        <is>
-          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="32" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>全国渠道</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>WinMart默认门店（待固定城市）</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>WinMart</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>Masan</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>MEATDeli</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>五花肉</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
-        </is>
-      </c>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>冷鲜</t>
-        </is>
-      </c>
-      <c r="I14" s="7" t="n">
-        <v>385</v>
-      </c>
-      <c r="J14" s="7" t="n">
-        <v>76962</v>
-      </c>
-      <c r="K14" s="7" t="n">
-        <v>199900</v>
-      </c>
-      <c r="L14" s="7" t="n"/>
-      <c r="M14" s="7">
-        <f>IF(L14&lt;&gt;"",L14,K14)</f>
-        <v/>
-      </c>
-      <c r="N14" s="5" t="inlineStr">
-        <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
-        </is>
-      </c>
-      <c r="O14" s="8" t="inlineStr">
         <is>
           <t>https://winmart.vn/products/meat-deli-ba-roi-heo--s10617959</t>
         </is>
@@ -1471,7 +1405,7 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M5:M14">
+  <conditionalFormatting sqref="M5:M13">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>150000</formula>
     </cfRule>
@@ -1489,7 +1423,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1604,7 +1537,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1646,7 +1579,7 @@
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>199900</v>
@@ -1688,7 +1621,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1856,7 +1789,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>138889</v>
@@ -1898,7 +1831,7 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>192100</v>
@@ -1940,7 +1873,7 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>138889</v>
@@ -1982,7 +1915,7 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F14" s="7" t="n">
         <v>165000</v>
@@ -2024,7 +1957,7 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>190000</v>
@@ -2066,7 +1999,7 @@
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F16" s="7" t="n">
         <v>197500</v>
@@ -2290,7 +2223,7 @@
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-nac-vai-heo-s--s10140279</t>
+          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-09-13
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-09-13</t>
+          <t>越南猪肉零售价格日报｜2026-09-14</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 06:23。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 06:32。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>9条在售商品</t>
+          <t>7条在售商品</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O13"/>
+  <dimension ref="A1:O11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-09-13</t>
+          <t>越南猪肉零售明细｜2026-09-14</t>
         </is>
       </c>
     </row>
@@ -1000,7 +1000,7 @@
       </c>
       <c r="O7" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g-ol341387</t>
+          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g</t>
         </is>
       </c>
     </row>
@@ -1066,7 +1066,7 @@
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g-ol341387</t>
+          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo Vĩnh Tân khay 200g</t>
+          <t>Nạc dăm heo Vĩnh Tân 400g</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -1112,13 +1112,13 @@
         </is>
       </c>
       <c r="I9" s="7" t="n">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>38000</v>
+        <v>77000</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>190000</v>
+        <v>192500</v>
       </c>
       <c r="L9" s="7" t="n"/>
       <c r="M9" s="7">
@@ -1132,7 +1132,7 @@
       </c>
       <c r="O9" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-400g-1-khay-63124</t>
         </is>
       </c>
     </row>
@@ -1205,37 +1205,37 @@
     <row r="11" ht="32" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>南部</t>
+          <t>全国渠道</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
+          <t>WinMart默认门店（待固定城市）</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>Masan</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>MEATDeli</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>小排</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Nạc đùi heo cắt xào Vĩnh Tân khay 200g</t>
+          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
@@ -1244,13 +1244,13 @@
         </is>
       </c>
       <c r="I11" s="7" t="n">
-        <v>200</v>
+        <v>431</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>33000</v>
+        <v>124085</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>165000</v>
+        <v>287900</v>
       </c>
       <c r="L11" s="7" t="n"/>
       <c r="M11" s="7">
@@ -1259,144 +1259,12 @@
       </c>
       <c r="N11" s="5" t="inlineStr">
         <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+          <t>中：官方交易页，但尚未固定配送门店</t>
         </is>
       </c>
       <c r="O11" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dui-heo-cat-xao-vinh-tan-khay-200g</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="32" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>全国渠道</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>WinMart默认门店（待固定城市）</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>WinMart</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Masan</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>MEATDeli</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>小排</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
-        </is>
-      </c>
-      <c r="H12" s="5" t="inlineStr">
-        <is>
-          <t>冷鲜</t>
-        </is>
-      </c>
-      <c r="I12" s="7" t="n">
-        <v>431</v>
-      </c>
-      <c r="J12" s="7" t="n">
-        <v>124085</v>
-      </c>
-      <c r="K12" s="7" t="n">
-        <v>287900</v>
-      </c>
-      <c r="L12" s="7" t="n"/>
-      <c r="M12" s="7">
-        <f>IF(L12&lt;&gt;"",L12,K12)</f>
-        <v/>
-      </c>
-      <c r="N12" s="5" t="inlineStr">
-        <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
-        </is>
-      </c>
-      <c r="O12" s="8" t="inlineStr">
-        <is>
           <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>全国渠道</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>WinMart默认门店（待固定城市）</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>WinMart</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Masan</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>MEATDeli</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>五花肉</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
-        </is>
-      </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>冷鲜</t>
-        </is>
-      </c>
-      <c r="I13" s="7" t="n">
-        <v>385</v>
-      </c>
-      <c r="J13" s="7" t="n">
-        <v>76962</v>
-      </c>
-      <c r="K13" s="7" t="n">
-        <v>199900</v>
-      </c>
-      <c r="L13" s="7" t="n"/>
-      <c r="M13" s="7">
-        <f>IF(L13&lt;&gt;"",L13,K13)</f>
-        <v/>
-      </c>
-      <c r="N13" s="5" t="inlineStr">
-        <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
-        </is>
-      </c>
-      <c r="O13" s="8" t="inlineStr">
-        <is>
-          <t>https://winmart.vn/products/meat-deli-ba-roi-heo--s10617959</t>
         </is>
       </c>
     </row>
@@ -1405,7 +1273,7 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M5:M13">
+  <conditionalFormatting sqref="M5:M11">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>150000</formula>
     </cfRule>
@@ -1421,8 +1289,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1537,7 +1403,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1621,7 +1487,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1789,7 +1655,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>138889</v>
@@ -1831,7 +1697,7 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>192100</v>
@@ -1873,7 +1739,7 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>138889</v>
@@ -1957,13 +1823,13 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>190000</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>190000</v>
+        <v>192500</v>
       </c>
       <c r="H15" s="7" t="n">
         <v>190000</v>
@@ -1999,7 +1865,7 @@
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F16" s="7" t="n">
         <v>197500</v>
@@ -2191,7 +2057,7 @@
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-400g-1-khay-63124</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-09-19
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-09-14</t>
+          <t>越南猪肉零售价格日报｜2026-09-20</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 06:32。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 06:34。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>7条在售商品</t>
+          <t>6条在售商品</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -610,12 +610,12 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>4个</t>
+          <t>2个</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>BAF、MEATDeli、Meatcool、Vĩnh Tân</t>
+          <t>MEATDeli、Meatcool</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O11"/>
+  <dimension ref="A1:O10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-09-14</t>
+          <t>越南猪肉零售明细｜2026-09-20</t>
         </is>
       </c>
     </row>
@@ -832,12 +832,12 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo Meatcool 360-440g</t>
+          <t>Cốt lết Meatcool 9-10 miếng/túi 900g</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
@@ -846,17 +846,15 @@
         </is>
       </c>
       <c r="I5" s="7" t="n">
-        <v>400</v>
+        <v>900</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>90400</v>
+        <v>125000</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>226000</v>
-      </c>
-      <c r="L5" s="7" t="n">
-        <v>192100</v>
-      </c>
+        <v>138889</v>
+      </c>
+      <c r="L5" s="7" t="n"/>
       <c r="M5" s="7">
         <f>IF(L5&lt;&gt;"",L5,K5)</f>
         <v/>
@@ -868,7 +866,7 @@
       </c>
       <c r="O5" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-meatcool-400g</t>
+          <t>https://kingfoodmart.com/thit-heo/sap-mo-ban-cot-let-meatcool-tui-900g-ol341387</t>
         </is>
       </c>
     </row>
@@ -890,22 +888,22 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>BAF</t>
+          <t>GREENFEED</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>BAF</t>
+          <t>Meatcool</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo BAF khay 300g</t>
+          <t>Thịt đùi Meatcool túi 900g</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
@@ -914,13 +912,13 @@
         </is>
       </c>
       <c r="I6" s="7" t="n">
-        <v>300</v>
+        <v>900</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>74000</v>
+        <v>125000</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>246667</v>
+        <v>138889</v>
       </c>
       <c r="L6" s="7" t="n"/>
       <c r="M6" s="7">
@@ -934,44 +932,44 @@
       </c>
       <c r="O6" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-baf-khay-300g-1-khay</t>
+          <t>https://kingfoodmart.com/thit-heo/sap-mo-ban-thit-dui-meatcool-tui-900g-ol341387</t>
         </is>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>南部</t>
+          <t>全国渠道</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
+          <t>WinMart默认门店（待固定城市）</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>GREENFEED</t>
+          <t>Masan</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>MEATDeli</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>肩肉</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Cốt lết Meatcool 9-10 miếng/túi 900g</t>
+          <t>MEATDELI Thịt Nạc vai heo (S)</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -980,13 +978,13 @@
         </is>
       </c>
       <c r="I7" s="7" t="n">
-        <v>900</v>
+        <v>440</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>125000</v>
+        <v>74316</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>138889</v>
+        <v>168900</v>
       </c>
       <c r="L7" s="7" t="n"/>
       <c r="M7" s="7">
@@ -995,49 +993,49 @@
       </c>
       <c r="N7" s="5" t="inlineStr">
         <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+          <t>中：官方交易页，但尚未固定配送门店</t>
         </is>
       </c>
       <c r="O7" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g</t>
+          <t>https://winmart.vn/products/meat-deli-nac-vai-heo-s--s10140279</t>
         </is>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>南部</t>
+          <t>全国渠道</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
+          <t>WinMart默认门店（待固定城市）</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>GREENFEED</t>
+          <t>Masan</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>MEATDeli</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>小排</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Thịt đùi Meatcool túi 900g</t>
+          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
@@ -1046,13 +1044,13 @@
         </is>
       </c>
       <c r="I8" s="7" t="n">
-        <v>900</v>
+        <v>431</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>125000</v>
+        <v>124085</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>138889</v>
+        <v>287900</v>
       </c>
       <c r="L8" s="7" t="n"/>
       <c r="M8" s="7">
@@ -1061,39 +1059,39 @@
       </c>
       <c r="N8" s="5" t="inlineStr">
         <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+          <t>中：官方交易页，但尚未固定配送门店</t>
         </is>
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
+          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
         </is>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>南部</t>
+          <t>全国渠道</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
+          <t>WinMart默认门店（待固定城市）</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>Masan</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>MEATDeli</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
@@ -1103,7 +1101,7 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo Vĩnh Tân 400g</t>
+          <t>MEATDELI Thịt Nạc dăm heo (Thịt Nạc vai) (S)</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -1115,10 +1113,10 @@
         <v>400</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>77000</v>
+        <v>81960</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>192500</v>
+        <v>204900</v>
       </c>
       <c r="L9" s="7" t="n"/>
       <c r="M9" s="7">
@@ -1127,49 +1125,49 @@
       </c>
       <c r="N9" s="5" t="inlineStr">
         <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+          <t>中：官方交易页，但尚未固定配送门店</t>
         </is>
       </c>
       <c r="O9" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-400g-1-khay-63124</t>
+          <t>https://winmart.vn/products/meat-deli-nac-dam-heo--s10617957</t>
         </is>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>南部</t>
+          <t>全国渠道</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
+          <t>WinMart默认门店（待固定城市）</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>Masan</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>MEATDeli</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>五花肉</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Nạc cốt lết cắt Vĩnh Tân khay 400g</t>
+          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
@@ -1178,13 +1176,13 @@
         </is>
       </c>
       <c r="I10" s="7" t="n">
-        <v>400</v>
+        <v>385</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>79000</v>
+        <v>76962</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>197500</v>
+        <v>199900</v>
       </c>
       <c r="L10" s="7" t="n"/>
       <c r="M10" s="7">
@@ -1193,78 +1191,12 @@
       </c>
       <c r="N10" s="5" t="inlineStr">
         <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+          <t>中：官方交易页，但尚未固定配送门店</t>
         </is>
       </c>
       <c r="O10" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="32" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>全国渠道</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>WinMart默认门店（待固定城市）</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>WinMart</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Masan</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>MEATDeli</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>小排</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
-        </is>
-      </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>冷鲜</t>
-        </is>
-      </c>
-      <c r="I11" s="7" t="n">
-        <v>431</v>
-      </c>
-      <c r="J11" s="7" t="n">
-        <v>124085</v>
-      </c>
-      <c r="K11" s="7" t="n">
-        <v>287900</v>
-      </c>
-      <c r="L11" s="7" t="n"/>
-      <c r="M11" s="7">
-        <f>IF(L11&lt;&gt;"",L11,K11)</f>
-        <v/>
-      </c>
-      <c r="N11" s="5" t="inlineStr">
-        <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
-        </is>
-      </c>
-      <c r="O11" s="8" t="inlineStr">
-        <is>
-          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
+          <t>https://winmart.vn/products/meat-deli-ba-roi-heo--s10617959</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1205,7 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M5:M11">
+  <conditionalFormatting sqref="M5:M10">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>150000</formula>
     </cfRule>
@@ -1288,7 +1220,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1445,7 +1376,7 @@
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>199900</v>
@@ -1487,7 +1418,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1529,7 +1460,7 @@
         </is>
       </c>
       <c r="E8" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F8" s="7" t="n">
         <v>204900</v>
@@ -1571,7 +1502,7 @@
         </is>
       </c>
       <c r="E9" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F9" s="7" t="n">
         <v>168900</v>
@@ -1655,7 +1586,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>138889</v>
@@ -1739,7 +1670,7 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>138889</v>
@@ -1908,7 +1839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1993,24 +1924,24 @@
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-meatcool-400g</t>
+          <t>https://kingfoodmart.com/thit-heo/sap-mo-ban-cot-let-meatcool-tui-900g-ol341387</t>
         </is>
       </c>
     </row>
     <row r="6" ht="58" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>BAF / BAF</t>
+          <t>Masan / MEATDeli</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>A-零售交易页</t>
+          <t>A-官方交易页</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -2020,76 +1951,12 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+          <t>中：官方交易页，但尚未固定配送门店</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-baf-khay-300g-1-khay</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="58" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Kingfoodmart</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Vĩnh Tân / Vĩnh Tân</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>A-零售交易页</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>实际价/kg = 促销价/kg（如有），否则常规价/kg；包装价÷重量(kg)用于交叉核验。</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
-        </is>
-      </c>
-      <c r="F7" s="8" t="inlineStr">
-        <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-400g-1-khay-63124</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="58" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>WinMart</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Masan / MEATDeli</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>A-官方交易页</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>实际价/kg = 促销价/kg（如有），否则常规价/kg；包装价÷重量(kg)用于交叉核验。</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
-        </is>
-      </c>
-      <c r="F8" s="8" t="inlineStr">
-        <is>
-          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
+          <t>https://winmart.vn/products/meat-deli-nac-vai-heo-s--s10140279</t>
         </is>
       </c>
     </row>
@@ -2101,8 +1968,6 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-09-20
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-09-20</t>
+          <t>越南猪肉零售价格日报｜2026-09-21</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 06:34。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 06:32。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>6条在售商品</t>
+          <t>5条在售商品</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O10"/>
+  <dimension ref="A1:O9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-09-20</t>
+          <t>越南猪肉零售明细｜2026-09-21</t>
         </is>
       </c>
     </row>
@@ -866,7 +866,7 @@
       </c>
       <c r="O5" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/sap-mo-ban-cot-let-meatcool-tui-900g-ol341387</t>
+          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g</t>
         </is>
       </c>
     </row>
@@ -932,7 +932,7 @@
       </c>
       <c r="O6" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/sap-mo-ban-thit-dui-meatcool-tui-900g-ol341387</t>
+          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
         </is>
       </c>
     </row>
@@ -964,12 +964,12 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>肩肉</t>
+          <t>小排</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI Thịt Nạc vai heo (S)</t>
+          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -978,13 +978,13 @@
         </is>
       </c>
       <c r="I7" s="7" t="n">
-        <v>440</v>
+        <v>431</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>74316</v>
+        <v>124085</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>168900</v>
+        <v>287900</v>
       </c>
       <c r="L7" s="7" t="n"/>
       <c r="M7" s="7">
@@ -998,7 +998,7 @@
       </c>
       <c r="O7" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-nac-vai-heo-s--s10140279</t>
+          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
         </is>
       </c>
     </row>
@@ -1030,12 +1030,12 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>小排</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
+          <t>MEATDELI Thịt Nạc dăm heo (Thịt Nạc vai) (S)</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
@@ -1044,13 +1044,13 @@
         </is>
       </c>
       <c r="I8" s="7" t="n">
-        <v>431</v>
+        <v>400</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>124085</v>
+        <v>81960</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>287900</v>
+        <v>204900</v>
       </c>
       <c r="L8" s="7" t="n"/>
       <c r="M8" s="7">
@@ -1064,7 +1064,7 @@
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
+          <t>https://winmart.vn/products/meat-deli-nac-dam-heo--s10617957</t>
         </is>
       </c>
     </row>
@@ -1096,12 +1096,12 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>五花肉</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI Thịt Nạc dăm heo (Thịt Nạc vai) (S)</t>
+          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -1110,13 +1110,13 @@
         </is>
       </c>
       <c r="I9" s="7" t="n">
-        <v>400</v>
+        <v>385</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>81960</v>
+        <v>76962</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>204900</v>
+        <v>199900</v>
       </c>
       <c r="L9" s="7" t="n"/>
       <c r="M9" s="7">
@@ -1129,72 +1129,6 @@
         </is>
       </c>
       <c r="O9" s="8" t="inlineStr">
-        <is>
-          <t>https://winmart.vn/products/meat-deli-nac-dam-heo--s10617957</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="32" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>全国渠道</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>WinMart默认门店（待固定城市）</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>WinMart</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Masan</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>MEATDeli</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>五花肉</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
-        </is>
-      </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>冷鲜</t>
-        </is>
-      </c>
-      <c r="I10" s="7" t="n">
-        <v>385</v>
-      </c>
-      <c r="J10" s="7" t="n">
-        <v>76962</v>
-      </c>
-      <c r="K10" s="7" t="n">
-        <v>199900</v>
-      </c>
-      <c r="L10" s="7" t="n"/>
-      <c r="M10" s="7">
-        <f>IF(L10&lt;&gt;"",L10,K10)</f>
-        <v/>
-      </c>
-      <c r="N10" s="5" t="inlineStr">
-        <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
-        </is>
-      </c>
-      <c r="O10" s="8" t="inlineStr">
         <is>
           <t>https://winmart.vn/products/meat-deli-ba-roi-heo--s10617959</t>
         </is>
@@ -1205,7 +1139,7 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M5:M10">
+  <conditionalFormatting sqref="M5:M9">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>150000</formula>
     </cfRule>
@@ -1219,7 +1153,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1376,7 +1309,7 @@
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>199900</v>
@@ -1418,7 +1351,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1460,7 +1393,7 @@
         </is>
       </c>
       <c r="E8" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F8" s="7" t="n">
         <v>204900</v>
@@ -1586,7 +1519,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>138889</v>
@@ -1670,7 +1603,7 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>138889</v>
@@ -1924,7 +1857,7 @@
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/sap-mo-ban-cot-let-meatcool-tui-900g-ol341387</t>
+          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g</t>
         </is>
       </c>
     </row>
@@ -1956,7 +1889,7 @@
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-nac-vai-heo-s--s10140279</t>
+          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-09-22
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-09-21</t>
+          <t>越南猪肉零售价格日报｜2026-09-22</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 06:32。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 07:17。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-09-21</t>
+          <t>越南猪肉零售明细｜2026-09-22</t>
         </is>
       </c>
     </row>
@@ -1309,7 +1309,7 @@
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>199900</v>
@@ -1351,7 +1351,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1393,7 +1393,7 @@
         </is>
       </c>
       <c r="E8" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F8" s="7" t="n">
         <v>204900</v>
@@ -1519,7 +1519,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>138889</v>
@@ -1603,7 +1603,7 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>138889</v>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-09-23
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-09-23</t>
+          <t>越南猪肉零售价格日报｜2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 06:50。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 06:58。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-09-23</t>
+          <t>越南猪肉零售明细｜2026-09-24</t>
         </is>
       </c>
     </row>
@@ -1376,7 +1376,7 @@
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>199900</v>
@@ -1418,7 +1418,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="E8" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F8" s="7" t="n">
         <v>204900</v>
@@ -1502,7 +1502,7 @@
         </is>
       </c>
       <c r="E9" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F9" s="7" t="n">
         <v>168900</v>
@@ -1586,7 +1586,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>138889</v>
@@ -1670,7 +1670,7 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>138889</v>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-09-25
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-09-24</t>
+          <t>越南猪肉零售价格日报｜2026-09-25</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 06:58。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 07:00。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-09-24</t>
+          <t>越南猪肉零售明细｜2026-09-25</t>
         </is>
       </c>
     </row>
@@ -1376,7 +1376,7 @@
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>199900</v>
@@ -1418,7 +1418,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="E8" s="7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F8" s="7" t="n">
         <v>204900</v>
@@ -1502,7 +1502,7 @@
         </is>
       </c>
       <c r="E9" s="7" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F9" s="7" t="n">
         <v>168900</v>
@@ -1586,7 +1586,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>138889</v>
@@ -1670,7 +1670,7 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>138889</v>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-09-26
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-09-25</t>
+          <t>越南猪肉零售价格日报｜2026-09-26</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 07:00。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 07:10。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>6条在售商品</t>
+          <t>7条在售商品</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O10"/>
+  <dimension ref="A1:O11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-09-25</t>
+          <t>越南猪肉零售明细｜2026-09-26</t>
         </is>
       </c>
     </row>
@@ -832,12 +832,12 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>五花肉</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Cốt lết Meatcool 9-10 miếng/túi 900g</t>
+          <t>Ba rọi heo Meatcool 350-450g</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
@@ -846,15 +846,17 @@
         </is>
       </c>
       <c r="I5" s="7" t="n">
-        <v>900</v>
+        <v>400</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>125000</v>
+        <v>99600</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>138889</v>
-      </c>
-      <c r="L5" s="7" t="n"/>
+        <v>249000</v>
+      </c>
+      <c r="L5" s="7" t="n">
+        <v>197500</v>
+      </c>
       <c r="M5" s="7">
         <f>IF(L5&lt;&gt;"",L5,K5)</f>
         <v/>
@@ -866,7 +868,7 @@
       </c>
       <c r="O5" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g</t>
+          <t>https://kingfoodmart.com/thit-heo/ba-roi-heo-meatcool-400g</t>
         </is>
       </c>
     </row>
@@ -898,12 +900,12 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Thịt đùi Meatcool túi 900g</t>
+          <t>Cốt lết Meatcool 9-10 miếng/túi 900g</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
@@ -932,44 +934,44 @@
       </c>
       <c r="O6" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
+          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g</t>
         </is>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>全国渠道</t>
+          <t>南部</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>WinMart默认门店（待固定城市）</t>
+          <t>胡志明市/Kingfoodmart默认门店</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>WinMart</t>
+          <t>Kingfoodmart</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Masan</t>
+          <t>GREENFEED</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>MEATDeli</t>
+          <t>Meatcool</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>肩肉</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI Thịt Nạc vai heo (S)</t>
+          <t>Thịt đùi Meatcool túi 900g</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -978,13 +980,13 @@
         </is>
       </c>
       <c r="I7" s="7" t="n">
-        <v>440</v>
+        <v>900</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>74316</v>
+        <v>125000</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>168900</v>
+        <v>138889</v>
       </c>
       <c r="L7" s="7" t="n"/>
       <c r="M7" s="7">
@@ -993,12 +995,12 @@
       </c>
       <c r="N7" s="5" t="inlineStr">
         <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
+          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
         </is>
       </c>
       <c r="O7" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-nac-vai-heo-s--s10140279</t>
+          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
         </is>
       </c>
     </row>
@@ -1030,12 +1032,12 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>小排</t>
+          <t>肩肉</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
+          <t>MEATDELI Thịt Nạc vai heo (S)</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
@@ -1044,13 +1046,13 @@
         </is>
       </c>
       <c r="I8" s="7" t="n">
-        <v>431</v>
+        <v>440</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>124085</v>
+        <v>74316</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>287900</v>
+        <v>168900</v>
       </c>
       <c r="L8" s="7" t="n"/>
       <c r="M8" s="7">
@@ -1064,7 +1066,7 @@
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
+          <t>https://winmart.vn/products/meat-deli-nac-vai-heo-s--s10140279</t>
         </is>
       </c>
     </row>
@@ -1096,12 +1098,12 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>小排</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI Thịt Nạc dăm heo (Thịt Nạc vai) (S)</t>
+          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -1110,13 +1112,13 @@
         </is>
       </c>
       <c r="I9" s="7" t="n">
-        <v>400</v>
+        <v>431</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>81960</v>
+        <v>124085</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>204900</v>
+        <v>287900</v>
       </c>
       <c r="L9" s="7" t="n"/>
       <c r="M9" s="7">
@@ -1130,7 +1132,7 @@
       </c>
       <c r="O9" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-nac-dam-heo--s10617957</t>
+          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
         </is>
       </c>
     </row>
@@ -1162,12 +1164,12 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>五花肉</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
+          <t>MEATDELI Thịt Nạc dăm heo (Thịt Nạc vai) (S)</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
@@ -1176,13 +1178,13 @@
         </is>
       </c>
       <c r="I10" s="7" t="n">
-        <v>385</v>
+        <v>400</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>76962</v>
+        <v>81960</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>199900</v>
+        <v>204900</v>
       </c>
       <c r="L10" s="7" t="n"/>
       <c r="M10" s="7">
@@ -1195,6 +1197,72 @@
         </is>
       </c>
       <c r="O10" s="8" t="inlineStr">
+        <is>
+          <t>https://winmart.vn/products/meat-deli-nac-dam-heo--s10617957</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>全国渠道</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>WinMart默认门店（待固定城市）</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>WinMart</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Masan</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>MEATDeli</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>五花肉</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>冷鲜</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="n">
+        <v>385</v>
+      </c>
+      <c r="J11" s="7" t="n">
+        <v>76962</v>
+      </c>
+      <c r="K11" s="7" t="n">
+        <v>199900</v>
+      </c>
+      <c r="L11" s="7" t="n"/>
+      <c r="M11" s="7">
+        <f>IF(L11&lt;&gt;"",L11,K11)</f>
+        <v/>
+      </c>
+      <c r="N11" s="5" t="inlineStr">
+        <is>
+          <t>中：官方交易页，但尚未固定配送门店</t>
+        </is>
+      </c>
+      <c r="O11" s="8" t="inlineStr">
         <is>
           <t>https://winmart.vn/products/meat-deli-ba-roi-heo--s10617959</t>
         </is>
@@ -1205,7 +1273,7 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M5:M10">
+  <conditionalFormatting sqref="M5:M11">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>150000</formula>
     </cfRule>
@@ -1220,6 +1288,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1376,7 +1445,7 @@
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>199900</v>
@@ -1418,7 +1487,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1460,7 +1529,7 @@
         </is>
       </c>
       <c r="E8" s="7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F8" s="7" t="n">
         <v>204900</v>
@@ -1502,7 +1571,7 @@
         </is>
       </c>
       <c r="E9" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F9" s="7" t="n">
         <v>168900</v>
@@ -1544,7 +1613,7 @@
         </is>
       </c>
       <c r="E10" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F10" s="7" t="n">
         <v>175555</v>
@@ -1586,7 +1655,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>138889</v>
@@ -1670,7 +1739,7 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>138889</v>
@@ -1924,7 +1993,7 @@
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g</t>
+          <t>https://kingfoodmart.com/thit-heo/ba-roi-heo-meatcool-400g</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-09-28
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-09-27</t>
+          <t>越南猪肉零售价格日报｜2026-09-28</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 06:55。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 08:11。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -588,12 +588,12 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>7条在售商品</t>
+          <t>3条在售商品</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>渠道：Kingfoodmart、WinMart</t>
+          <t>渠道：WinMart</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -610,12 +610,12 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>2个</t>
+          <t>1个</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>MEATDeli、Meatcool</t>
+          <t>MEATDeli</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O11"/>
+  <dimension ref="A1:O7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-09-27</t>
+          <t>越南猪肉零售明细｜2026-09-28</t>
         </is>
       </c>
     </row>
@@ -807,37 +807,37 @@
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>南部</t>
+          <t>全国渠道</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
+          <t>WinMart默认门店（待固定城市）</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>GREENFEED</t>
+          <t>Masan</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>MEATDeli</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>五花肉</t>
+          <t>小排</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Ba rọi heo Meatcool 350-450g</t>
+          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
@@ -846,66 +846,64 @@
         </is>
       </c>
       <c r="I5" s="7" t="n">
-        <v>400</v>
+        <v>431</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>99600</v>
+        <v>124085</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>249000</v>
-      </c>
-      <c r="L5" s="7" t="n">
-        <v>197500</v>
-      </c>
+        <v>287900</v>
+      </c>
+      <c r="L5" s="7" t="n"/>
       <c r="M5" s="7">
         <f>IF(L5&lt;&gt;"",L5,K5)</f>
         <v/>
       </c>
       <c r="N5" s="5" t="inlineStr">
         <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+          <t>中：官方交易页，但尚未固定配送门店</t>
         </is>
       </c>
       <c r="O5" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/ba-roi-heo-meatcool-400g</t>
+          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
         </is>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>南部</t>
+          <t>全国渠道</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
+          <t>WinMart默认门店（待固定城市）</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>GREENFEED</t>
+          <t>Masan</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>MEATDeli</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Cốt lết Meatcool 9-10 miếng/túi 900g</t>
+          <t>MEATDELI Thịt Nạc dăm heo (Thịt Nạc vai) (S)</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
@@ -914,13 +912,13 @@
         </is>
       </c>
       <c r="I6" s="7" t="n">
-        <v>900</v>
+        <v>400</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>125000</v>
+        <v>81960</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>138889</v>
+        <v>204900</v>
       </c>
       <c r="L6" s="7" t="n"/>
       <c r="M6" s="7">
@@ -929,49 +927,49 @@
       </c>
       <c r="N6" s="5" t="inlineStr">
         <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+          <t>中：官方交易页，但尚未固定配送门店</t>
         </is>
       </c>
       <c r="O6" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g</t>
+          <t>https://winmart.vn/products/meat-deli-nac-dam-heo--s10617957</t>
         </is>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>南部</t>
+          <t>全国渠道</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
+          <t>WinMart默认门店（待固定城市）</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>GREENFEED</t>
+          <t>Masan</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>MEATDeli</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>五花肉</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Thịt đùi Meatcool túi 900g</t>
+          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -980,13 +978,13 @@
         </is>
       </c>
       <c r="I7" s="7" t="n">
-        <v>900</v>
+        <v>385</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>125000</v>
+        <v>76962</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>138889</v>
+        <v>199900</v>
       </c>
       <c r="L7" s="7" t="n"/>
       <c r="M7" s="7">
@@ -995,274 +993,10 @@
       </c>
       <c r="N7" s="5" t="inlineStr">
         <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+          <t>中：官方交易页，但尚未固定配送门店</t>
         </is>
       </c>
       <c r="O7" s="8" t="inlineStr">
-        <is>
-          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="32" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>全国渠道</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>WinMart默认门店（待固定城市）</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>WinMart</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Masan</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>MEATDeli</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>肩肉</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>MEATDELI Thịt Nạc vai heo (S)</t>
-        </is>
-      </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>冷鲜</t>
-        </is>
-      </c>
-      <c r="I8" s="7" t="n">
-        <v>440</v>
-      </c>
-      <c r="J8" s="7" t="n">
-        <v>74316</v>
-      </c>
-      <c r="K8" s="7" t="n">
-        <v>168900</v>
-      </c>
-      <c r="L8" s="7" t="n"/>
-      <c r="M8" s="7">
-        <f>IF(L8&lt;&gt;"",L8,K8)</f>
-        <v/>
-      </c>
-      <c r="N8" s="5" t="inlineStr">
-        <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
-        </is>
-      </c>
-      <c r="O8" s="8" t="inlineStr">
-        <is>
-          <t>https://winmart.vn/products/meat-deli-nac-vai-heo-s--s10140279</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="32" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>全国渠道</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>WinMart默认门店（待固定城市）</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>WinMart</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Masan</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>MEATDeli</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>小排</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>冷鲜</t>
-        </is>
-      </c>
-      <c r="I9" s="7" t="n">
-        <v>431</v>
-      </c>
-      <c r="J9" s="7" t="n">
-        <v>124085</v>
-      </c>
-      <c r="K9" s="7" t="n">
-        <v>287900</v>
-      </c>
-      <c r="L9" s="7" t="n"/>
-      <c r="M9" s="7">
-        <f>IF(L9&lt;&gt;"",L9,K9)</f>
-        <v/>
-      </c>
-      <c r="N9" s="5" t="inlineStr">
-        <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
-        </is>
-      </c>
-      <c r="O9" s="8" t="inlineStr">
-        <is>
-          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="32" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>全国渠道</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>WinMart默认门店（待固定城市）</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>WinMart</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Masan</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>MEATDeli</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>梅花肉</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>MEATDELI Thịt Nạc dăm heo (Thịt Nạc vai) (S)</t>
-        </is>
-      </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>冷鲜</t>
-        </is>
-      </c>
-      <c r="I10" s="7" t="n">
-        <v>400</v>
-      </c>
-      <c r="J10" s="7" t="n">
-        <v>81960</v>
-      </c>
-      <c r="K10" s="7" t="n">
-        <v>204900</v>
-      </c>
-      <c r="L10" s="7" t="n"/>
-      <c r="M10" s="7">
-        <f>IF(L10&lt;&gt;"",L10,K10)</f>
-        <v/>
-      </c>
-      <c r="N10" s="5" t="inlineStr">
-        <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
-        </is>
-      </c>
-      <c r="O10" s="8" t="inlineStr">
-        <is>
-          <t>https://winmart.vn/products/meat-deli-nac-dam-heo--s10617957</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="32" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>全国渠道</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>WinMart默认门店（待固定城市）</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>WinMart</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Masan</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>MEATDeli</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>五花肉</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
-        </is>
-      </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>冷鲜</t>
-        </is>
-      </c>
-      <c r="I11" s="7" t="n">
-        <v>385</v>
-      </c>
-      <c r="J11" s="7" t="n">
-        <v>76962</v>
-      </c>
-      <c r="K11" s="7" t="n">
-        <v>199900</v>
-      </c>
-      <c r="L11" s="7" t="n"/>
-      <c r="M11" s="7">
-        <f>IF(L11&lt;&gt;"",L11,K11)</f>
-        <v/>
-      </c>
-      <c r="N11" s="5" t="inlineStr">
-        <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
-        </is>
-      </c>
-      <c r="O11" s="8" t="inlineStr">
         <is>
           <t>https://winmart.vn/products/meat-deli-ba-roi-heo--s10617959</t>
         </is>
@@ -1273,7 +1007,7 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M5:M11">
+  <conditionalFormatting sqref="M5:M7">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>150000</formula>
     </cfRule>
@@ -1285,10 +1019,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1445,7 +1175,7 @@
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>199900</v>
@@ -1487,7 +1217,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1529,7 +1259,7 @@
         </is>
       </c>
       <c r="E8" s="7" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F8" s="7" t="n">
         <v>204900</v>
@@ -1908,7 +1638,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1968,17 +1698,17 @@
     <row r="5" ht="58" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>GREENFEED / Meatcool</t>
+          <t>Masan / MEATDeli</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>A-零售交易页</t>
+          <t>A-官方交易页</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -1988,44 +1718,12 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+          <t>中：官方交易页，但尚未固定配送门店</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/ba-roi-heo-meatcool-400g</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="58" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>WinMart</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Masan / MEATDeli</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>A-官方交易页</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>实际价/kg = 促销价/kg（如有），否则常规价/kg；包装价÷重量(kg)用于交叉核验。</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
-        </is>
-      </c>
-      <c r="F6" s="8" t="inlineStr">
-        <is>
-          <t>https://winmart.vn/products/meat-deli-nac-vai-heo-s--s10140279</t>
+          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
         </is>
       </c>
     </row>
@@ -2036,7 +1734,6 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-09-29
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-09-28</t>
+          <t>越南猪肉零售价格日报｜2026-09-29</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 08:11。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 08:16。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -588,12 +588,12 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>3条在售商品</t>
+          <t>4条在售商品</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>渠道：WinMart</t>
+          <t>渠道：Kingfoodmart、WinMart</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -610,12 +610,12 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>1个</t>
+          <t>2个</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>MEATDeli</t>
+          <t>MEATDeli、Meatcool</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O7"/>
+  <dimension ref="A1:O8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-09-28</t>
+          <t>越南猪肉零售明细｜2026-09-29</t>
         </is>
       </c>
     </row>
@@ -807,37 +807,37 @@
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>全国渠道</t>
+          <t>南部</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>WinMart默认门店（待固定城市）</t>
+          <t>胡志明市/Kingfoodmart默认门店</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>WinMart</t>
+          <t>Kingfoodmart</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Masan</t>
+          <t>GREENFEED</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>MEATDeli</t>
+          <t>Meatcool</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>小排</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
+          <t>Cốt lết Meatcool 9-10 miếng/túi 900g</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
@@ -846,13 +846,13 @@
         </is>
       </c>
       <c r="I5" s="7" t="n">
-        <v>431</v>
+        <v>900</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>124085</v>
+        <v>125000</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>287900</v>
+        <v>138889</v>
       </c>
       <c r="L5" s="7" t="n"/>
       <c r="M5" s="7">
@@ -861,49 +861,49 @@
       </c>
       <c r="N5" s="5" t="inlineStr">
         <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
+          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
         </is>
       </c>
       <c r="O5" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
+          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g</t>
         </is>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>全国渠道</t>
+          <t>南部</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>WinMart默认门店（待固定城市）</t>
+          <t>胡志明市/Kingfoodmart默认门店</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>WinMart</t>
+          <t>Kingfoodmart</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Masan</t>
+          <t>GREENFEED</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>MEATDeli</t>
+          <t>Meatcool</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI Thịt Nạc dăm heo (Thịt Nạc vai) (S)</t>
+          <t>Thịt đùi Meatcool túi 900g</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
@@ -912,13 +912,13 @@
         </is>
       </c>
       <c r="I6" s="7" t="n">
-        <v>400</v>
+        <v>900</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>81960</v>
+        <v>125000</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>204900</v>
+        <v>138889</v>
       </c>
       <c r="L6" s="7" t="n"/>
       <c r="M6" s="7">
@@ -927,12 +927,12 @@
       </c>
       <c r="N6" s="5" t="inlineStr">
         <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
+          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
         </is>
       </c>
       <c r="O6" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-nac-dam-heo--s10617957</t>
+          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
         </is>
       </c>
     </row>
@@ -964,12 +964,12 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>五花肉</t>
+          <t>小排</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
+          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -978,13 +978,13 @@
         </is>
       </c>
       <c r="I7" s="7" t="n">
-        <v>385</v>
+        <v>431</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>76962</v>
+        <v>124085</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>199900</v>
+        <v>287900</v>
       </c>
       <c r="L7" s="7" t="n"/>
       <c r="M7" s="7">
@@ -997,6 +997,72 @@
         </is>
       </c>
       <c r="O7" s="8" t="inlineStr">
+        <is>
+          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="32" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>全国渠道</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>WinMart默认门店（待固定城市）</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>WinMart</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Masan</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>MEATDeli</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>五花肉</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>冷鲜</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="n">
+        <v>385</v>
+      </c>
+      <c r="J8" s="7" t="n">
+        <v>76962</v>
+      </c>
+      <c r="K8" s="7" t="n">
+        <v>199900</v>
+      </c>
+      <c r="L8" s="7" t="n"/>
+      <c r="M8" s="7">
+        <f>IF(L8&lt;&gt;"",L8,K8)</f>
+        <v/>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>中：官方交易页，但尚未固定配送门店</t>
+        </is>
+      </c>
+      <c r="O8" s="8" t="inlineStr">
         <is>
           <t>https://winmart.vn/products/meat-deli-ba-roi-heo--s10617959</t>
         </is>
@@ -1007,7 +1073,7 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M5:M7">
+  <conditionalFormatting sqref="M5:M8">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>150000</formula>
     </cfRule>
@@ -1019,6 +1085,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1175,7 +1242,7 @@
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>199900</v>
@@ -1217,7 +1284,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1385,7 +1452,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>138889</v>
@@ -1469,7 +1536,7 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>138889</v>
@@ -1638,7 +1705,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1698,30 +1765,62 @@
     <row r="5" ht="58" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
+          <t>Kingfoodmart</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>GREENFEED / Meatcool</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>A-零售交易页</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>实际价/kg = 促销价/kg（如有），否则常规价/kg；包装价÷重量(kg)用于交叉核验。</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="58" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
           <t>WinMart</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Masan / MEATDeli</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>A-官方交易页</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>实际价/kg = 促销价/kg（如有），否则常规价/kg；包装价÷重量(kg)用于交叉核验。</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>中：官方交易页，但尚未固定配送门店</t>
         </is>
       </c>
-      <c r="F5" s="8" t="inlineStr">
+      <c r="F6" s="8" t="inlineStr">
         <is>
           <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
         </is>
@@ -1734,6 +1833,7 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>